<commit_message>
Added sources for the population denominators plus additional notes/information. 2 data files for ethnic group populations also added to repo.
</commit_message>
<xml_diff>
--- a/data/cqc_metrics.xlsx
+++ b/data/cqc_metrics.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/ad-hoc/CQC SOC report/repo/cqc_soc/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{C106DA94-F57A-46FF-A4F8-71D897C3998A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E9066BF-800C-4C6D-B6D5-355F9BD8F429}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="8_{C106DA94-F57A-46FF-A4F8-71D897C3998A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A382EB8-7893-4D38-BBB7-EC80FB0E629B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1665" windowWidth="29040" windowHeight="15225" xr2:uid="{E0173AC4-6F6F-4158-8A16-D04BBE4744E4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="UEC" sheetId="1" r:id="rId1"/>
+    <sheet name="NHS111" sheetId="2" r:id="rId2"/>
+    <sheet name="code snippets" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="146">
   <si>
     <t>% MH arriving by ambulance/self</t>
   </si>
@@ -120,13 +122,367 @@
   </si>
   <si>
     <t>crude rate per 1,000 with relevant CI</t>
+  </si>
+  <si>
+    <t>https://www.ons.gov.uk/peoplepopulationandcommunity/populationandmigration/populationestimates/datasets/clinicalcommissioninggroupmidyearpopulationestimates</t>
+  </si>
+  <si>
+    <t>Source1</t>
+  </si>
+  <si>
+    <t>Source2</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>https://www.ons.gov.uk/peoplepopulationandcommunity/populationandmigration/populationestimates/datasets/lowersuperoutputareamidyearpopulationestimates</t>
+  </si>
+  <si>
+    <t>icb available 2022 and 2021. Prior years best to use lsoa pops aggregated to ICB (https://geoportal.statistics.gov.uk/datasets/423c8069710c4d488d5ff99475688101/explore)</t>
+  </si>
+  <si>
+    <t>wrangled</t>
+  </si>
+  <si>
+    <t>obtained</t>
+  </si>
+  <si>
+    <t>initial for completed</t>
+  </si>
+  <si>
+    <t>in repo</t>
+  </si>
+  <si>
+    <t>## ethnicity census imputed trends</t>
+  </si>
+  <si>
+    <t>ethnicity_icb_2011 &lt;- read.csv("repo/West_Midlands_Paediatric_Review/reference/ethnic_groups_LAD_2011_under25.csv") %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  clean_names() %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate_if(is.character, list(~na_if(.,""))) %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  select(lad11cd, lad21nm, region, icb22nm, white, asian, black, mixed, other) %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  rename(area_code = lad11cd, area_name = lad21nm) %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  filter(region %in% c("East Midlands","West Midlands")) %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  group_by(region, icb22nm) %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  summarise(across(c(3:7), ~ sum(., na.rm = TRUE))) %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(total = white+black+asian+mixed+other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ,der_financial_year = '2011/12')</t>
+  </si>
+  <si>
+    <t>ethnicity_icb_2021 &lt;- read.csv("repo/West_Midlands_Paediatric_Review/reference/ethnic_groups_LAD_2021_under25.csv") %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  select(lad21cd, lad21nm, region, icb22nm, white, asian, black, mixed, other) %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  rename(area_code = lad21cd, area_name = lad21nm) %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ,der_financial_year = '2021/22')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_both &lt;- ethnicity_icb_2011 %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  left_join(ethnicity_icb_2021, by = "icb22nm")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2012_13 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*1),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*1),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*1),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*1),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*1),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*1),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2012/13') %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  select(c(1:2,18:24)) %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  rename(region = region.x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2013_14 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*2),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*2),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*2),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*2),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*2),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*2),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2013/14') %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2014_15 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*3),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*3),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*3),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*3),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*3),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*3),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2014/15') %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2015_16 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*4),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*4),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*4),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*4),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*4),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*4),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2015/16') %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2016_17 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*5),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*5),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*5),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*5),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*5),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*5),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2016/17') %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2017_18 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*6),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*6),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*6),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*6),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*6),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*6),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2017/18') %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2018_19 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*7),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*7),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*7),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*7),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*7),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*7),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2018/19') %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2019_20 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*8),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*8),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*8),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*8),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*8),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*8),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2019/20') %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2020_21 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*9),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*9),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*9),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*9),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*9),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*9),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2020/21') %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2022_23 &lt;- ethnicity_icb_both %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  mutate(white = round(white.x + ((white.y-white.x)/10*11),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,asian = round(asian.x + ((asian.y-asian.x)/10*11),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,black = round(black.x + ((black.y-black.x)/10*11),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,mixed = round(mixed.x + ((mixed.y-mixed.x)/10*11),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,other = round(other.x + ((other.y-other.x)/10*11),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,total = round(total.x + ((total.y-total.x)/10*11),0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         ,der_financial_year = '2022/23') %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ethnicity_icb_2011_to_2022 &lt;- rbind(ethnicity_icb_2011, ethnicity_icb_2012_13, ethnicity_icb_2013_14, ethnicity_icb_2014_15, ethnicity_icb_2015_16, ethnicity_icb_2016_17, ethnicity_icb_2017_18, ethnicity_icb_2018_19, ethnicity_icb_2019_20, ethnicity_icb_2020_21, ethnicity_icb_2021, ethnicity_icb_2022_23) %&gt;% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  pivot_longer(!c(region, icb22nm, der_financial_year), names_to = 'ethnic_group', values_to = 'population')</t>
+  </si>
+  <si>
+    <t>rm(ethnicity_icb_2011, ethnicity_icb_2012_13, ethnicity_icb_2013_14, ethnicity_icb_2014_15, ethnicity_icb_2015_16, ethnicity_icb_2016_17, ethnicity_icb_2017_18, ethnicity_icb_2018_19, ethnicity_icb_2019_20, ethnicity_icb_2020_21, ethnicity_icb_2021, ethnicity_icb_2022_23, ethnicity_icb_both)</t>
+  </si>
+  <si>
+    <t>Ethnicity imputed by year (under 25s)</t>
+  </si>
+  <si>
+    <t>I did this for under 25's for the paeds project - snippet in this workbook - and have saved the all age equivalent files to the data folder in this repo. May also need to source a full LAD to ICB lookup as i only did for Midlands manually. Make this prettier and more efficient please 😁.</t>
+  </si>
+  <si>
+    <t>https://assets.publishing.service.gov.uk/media/5d8b3abded915d0373d3540f/File_1_-_IMD2019_Index_of_Multiple_Deprivation.xlsx</t>
+  </si>
+  <si>
+    <t>Apply (all age) lsoa pops by year to 2019 IMD deciles</t>
+  </si>
+  <si>
+    <t>https://www.gov.uk/government/statistics/2011-rural-urban-classification-lookup-tables-for-all-geographies</t>
+  </si>
+  <si>
+    <t>Apply (all age) lsoa pops by year to 2011 rural urban classification (2 category)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,6 +522,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -188,15 +559,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -532,162 +909,929 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E043F9F0-0DBA-4E8F-9109-A6A749EE8BC1}">
-  <dimension ref="A2:G21"/>
+  <dimension ref="A2:I22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="15.81640625" customWidth="1"/>
     <col min="3" max="3" width="34.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="38.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>21</v>
       </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>0</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B6" s="3" t="s">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F12" s="1" t="s">
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B13" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B14" s="4"/>
+      <c r="G14" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D15" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B16" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B17" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="5" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="B18" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="B19" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="B20" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D16" r:id="rId1" xr:uid="{11D6067B-A8E8-45DB-B183-F9A149027B92}"/>
+    <hyperlink ref="E16" r:id="rId2" xr:uid="{171B83D9-6216-4E69-B2EA-9CBC19E4A36D}"/>
+    <hyperlink ref="D17" r:id="rId3" xr:uid="{D42BD446-88BF-4F5A-A6A2-EAF9494FF80D}"/>
+    <hyperlink ref="E17" r:id="rId4" xr:uid="{091DCC6B-C431-46F9-8CD0-8CBE1F8127D5}"/>
+    <hyperlink ref="D19" r:id="rId5" xr:uid="{CAF6641D-1BEB-46D7-A18F-FA3FA25615E3}"/>
+    <hyperlink ref="E19" r:id="rId6" xr:uid="{60AD5DC8-5870-4485-9449-19048E8CCE84}"/>
+    <hyperlink ref="D20" r:id="rId7" xr:uid="{654D7616-7933-463E-A9B8-5C1D1C5C56E2}"/>
+    <hyperlink ref="E20" r:id="rId8" xr:uid="{23777C45-1E6F-4AD0-A9FC-E7A425AFC12B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{835B9890-ED73-4CF5-BE95-2A8A5BAE7287}">
+  <dimension ref="A2:C18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B10" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B13" s="5" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
-      </c>
-      <c r="F15" t="s">
-        <v>4</v>
-      </c>
-      <c r="G15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>17</v>
-      </c>
-      <c r="F16" t="s">
-        <v>3</v>
-      </c>
-      <c r="G16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4DE2C38-DB6E-43CC-9653-D659AD256797}">
+  <dimension ref="B2:B143"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="107.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" t="s">
-        <v>18</v>
-      </c>
-      <c r="F17" t="s">
-        <v>6</v>
-      </c>
-      <c r="G17" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" t="s">
-        <v>9</v>
-      </c>
-      <c r="G18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>23</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B28" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B30" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B31" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B32" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B34" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B35" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B36" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B37" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B38" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B41" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B42" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B43" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B44" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B45" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B46" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B47" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B48" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B49" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B50" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B52" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B53" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B54" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B55" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B56" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B57" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B58" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B59" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B60" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B61" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B63" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B64" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B65" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B66" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B67" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B68" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B69" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B70" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B71" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B72" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B74" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B75" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B76" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B77" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B78" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B79" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B80" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B81" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B82" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B83" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B85" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B86" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B87" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B88" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B89" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B90" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B91" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B92" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B93" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B94" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B96" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B97" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B98" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B99" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B100" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B101" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B102" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B103" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B104" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B105" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B107" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B108" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B109" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B110" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B111" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B112" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B113" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B114" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B115" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B116" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B118" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B119" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B120" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B121" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B122" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="123" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B123" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="124" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B124" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="125" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B125" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="126" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B126" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B127" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B129" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="130" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B130" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="131" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B131" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="132" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B132" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="133" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B133" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="134" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B134" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="135" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B135" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="136" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B136" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="137" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B137" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="138" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B138" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="140" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B140" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="141" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B141" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="143" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B143" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added a time in ED metric and adjusted age groups as per meeting with cqc
</commit_message>
<xml_diff>
--- a/data/cqc_metrics.xlsx
+++ b/data/cqc_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/anya_ferguson_mlcsu_nhs_uk/Documents/Documents/Files/Projects/active/cqc_soc/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/ad-hoc/CQC SOC report/repo/cqc_soc/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="99" documentId="8_{C106DA94-F57A-46FF-A4F8-71D897C3998A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67F91DEF-09BA-4A40-B0BA-EFB0B8C46464}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="114_{98E47C94-B35C-48A9-87FF-0894DDAB52FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D943ED8E-8BBC-4D3D-9E19-5B3219451D18}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="10360" xr2:uid="{E0173AC4-6F6F-4158-8A16-D04BBE4744E4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11000" xr2:uid="{E0173AC4-6F6F-4158-8A16-D04BBE4744E4}"/>
   </bookViews>
   <sheets>
     <sheet name="UEC" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="148">
   <si>
     <t>% MH arriving by ambulance/self</t>
   </si>
@@ -88,18 +88,12 @@
     <t>Call disposition of MH calls</t>
   </si>
   <si>
-    <t>0-19; 20-34; 35-59; 60-74; 75+</t>
-  </si>
-  <si>
     <t>male; female</t>
   </si>
   <si>
     <t>White; Mixed; Asian; Black; Other</t>
   </si>
   <si>
-    <t>Calls by chief complaint</t>
-  </si>
-  <si>
     <t>Call rates for any MH, sub-group analysis (all by ICB and year?)</t>
   </si>
   <si>
@@ -479,6 +473,15 @@
   </si>
   <si>
     <t>AF</t>
+  </si>
+  <si>
+    <t>Median/Mean time in ED department</t>
+  </si>
+  <si>
+    <t>0-17; 18-21; 22-39; 40-64; 65-74; 75+</t>
+  </si>
+  <si>
+    <t>Calls by symptom group</t>
   </si>
 </sst>
 </file>
@@ -912,7 +915,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E043F9F0-0DBA-4E8F-9109-A6A749EE8BC1}">
-  <dimension ref="A2:I22"/>
+  <dimension ref="A2:I23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="15.81640625" customWidth="1"/>
@@ -922,12 +925,12 @@
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -947,187 +950,195 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B12" s="1" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B13" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B13" s="4" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B14" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B15" s="4"/>
+      <c r="G15" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D16" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B14" s="4"/>
-      <c r="G14" s="7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="D15" t="s">
+      <c r="E16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" t="s">
         <v>29</v>
       </c>
-      <c r="E15" t="s">
-        <v>30</v>
-      </c>
-      <c r="F15" t="s">
-        <v>31</v>
-      </c>
-      <c r="G15" t="s">
+      <c r="G16" t="s">
+        <v>33</v>
+      </c>
+      <c r="H16" t="s">
+        <v>32</v>
+      </c>
+      <c r="I16" t="s">
         <v>35</v>
-      </c>
-      <c r="H15" t="s">
-        <v>34</v>
-      </c>
-      <c r="I15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B16" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B17" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B18" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C18" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" s="5" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="B19" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" s="5" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="B18" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
-      <c r="B19" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>142</v>
-      </c>
       <c r="F19" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:9" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="B20" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="B21" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E20" s="6" t="s">
+      <c r="C21" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="G21" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F20" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>23</v>
+      <c r="H21" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="D16" r:id="rId1" xr:uid="{11D6067B-A8E8-45DB-B183-F9A149027B92}"/>
-    <hyperlink ref="E16" r:id="rId2" xr:uid="{171B83D9-6216-4E69-B2EA-9CBC19E4A36D}"/>
-    <hyperlink ref="D17" r:id="rId3" xr:uid="{D42BD446-88BF-4F5A-A6A2-EAF9494FF80D}"/>
-    <hyperlink ref="E17" r:id="rId4" xr:uid="{091DCC6B-C431-46F9-8CD0-8CBE1F8127D5}"/>
-    <hyperlink ref="D19" r:id="rId5" xr:uid="{CAF6641D-1BEB-46D7-A18F-FA3FA25615E3}"/>
-    <hyperlink ref="E19" r:id="rId6" xr:uid="{60AD5DC8-5870-4485-9449-19048E8CCE84}"/>
-    <hyperlink ref="D20" r:id="rId7" xr:uid="{654D7616-7933-463E-A9B8-5C1D1C5C56E2}"/>
-    <hyperlink ref="E20" r:id="rId8" xr:uid="{23777C45-1E6F-4AD0-A9FC-E7A425AFC12B}"/>
+    <hyperlink ref="D17" r:id="rId1" xr:uid="{11D6067B-A8E8-45DB-B183-F9A149027B92}"/>
+    <hyperlink ref="E17" r:id="rId2" xr:uid="{171B83D9-6216-4E69-B2EA-9CBC19E4A36D}"/>
+    <hyperlink ref="D18" r:id="rId3" xr:uid="{D42BD446-88BF-4F5A-A6A2-EAF9494FF80D}"/>
+    <hyperlink ref="E18" r:id="rId4" xr:uid="{091DCC6B-C431-46F9-8CD0-8CBE1F8127D5}"/>
+    <hyperlink ref="D20" r:id="rId5" xr:uid="{CAF6641D-1BEB-46D7-A18F-FA3FA25615E3}"/>
+    <hyperlink ref="E20" r:id="rId6" xr:uid="{60AD5DC8-5870-4485-9449-19048E8CCE84}"/>
+    <hyperlink ref="D21" r:id="rId7" xr:uid="{654D7616-7933-463E-A9B8-5C1D1C5C56E2}"/>
+    <hyperlink ref="E21" r:id="rId8" xr:uid="{23777C45-1E6F-4AD0-A9FC-E7A425AFC12B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
@@ -1141,7 +1152,7 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -1161,15 +1172,15 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
@@ -1177,12 +1188,12 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B11" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -1193,7 +1204,7 @@
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -1201,7 +1212,7 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
@@ -1217,12 +1228,12 @@
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1240,637 +1251,637 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B37" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B38" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="41" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="42" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="43" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B43" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="44" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B44" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B45" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B46" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="47" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="48" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B48" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B49" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B50" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="52" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B52" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="53" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B53" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="54" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B55" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="56" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B56" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="57" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="59" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B59" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="60" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="61" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="63" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="64" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="65" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="71" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B71" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="72" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B72" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="74" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B74" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="75" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B75" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="76" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B76" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="77" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="78" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="79" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B81" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="82" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B82" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="83" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B83" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="85" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B85" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="86" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B86" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="87" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B87" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="88" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B88" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="89" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B89" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="90" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B90" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="91" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B91" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="92" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B92" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="93" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B93" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="94" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B94" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="96" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B96" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B97" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B98" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B99" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B100" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B101" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="102" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B102" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="103" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B103" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="104" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B104" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="105" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B105" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="107" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B107" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="108" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B108" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="109" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B109" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="110" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B110" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="111" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B111" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="112" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B112" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="113" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B113" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="114" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B114" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="115" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B115" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="116" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B116" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="118" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B118" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="119" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B119" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="120" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B120" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="121" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B121" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="122" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B122" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="123" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B123" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="124" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B124" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="125" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B125" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="126" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B126" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="127" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B127" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="129" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B129" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="130" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B130" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="131" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B131" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="132" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B132" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="133" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B133" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="134" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B134" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="135" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B135" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="136" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B136" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="137" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B137" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="138" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B138" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="140" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B140" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="141" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B141" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="143" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B143" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
exlcusions from snomed and 111 symptom lookups. Data files for specific queries
</commit_message>
<xml_diff>
--- a/data/cqc_metrics.xlsx
+++ b/data/cqc_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/ad-hoc/CQC SOC report/repo/cqc_soc/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="114_{98E47C94-B35C-48A9-87FF-0894DDAB52FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D943ED8E-8BBC-4D3D-9E19-5B3219451D18}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="114_{98E47C94-B35C-48A9-87FF-0894DDAB52FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15380AE6-8203-4C5A-979E-A8E01706C37F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11000" xr2:uid="{E0173AC4-6F6F-4158-8A16-D04BBE4744E4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11000" activeTab="1" xr2:uid="{E0173AC4-6F6F-4158-8A16-D04BBE4744E4}"/>
   </bookViews>
   <sheets>
     <sheet name="UEC" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="154">
   <si>
     <t>% MH arriving by ambulance/self</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Attendance rates for any MH, sub-group analysis (all by ICB and year?)</t>
   </si>
   <si>
-    <t>Attendances by MH reason (grouped)</t>
-  </si>
-  <si>
     <t>Rural-Urban</t>
   </si>
   <si>
@@ -482,6 +479,27 @@
   </si>
   <si>
     <t>Calls by symptom group</t>
+  </si>
+  <si>
+    <t>extracted to data folder - ae_waits_icb.csv</t>
+  </si>
+  <si>
+    <t>extracted to data folder - ae_freqfly_icb.csv</t>
+  </si>
+  <si>
+    <t>Attendances by MH reason SNOMED</t>
+  </si>
+  <si>
+    <t>extracted to data folder - ae_diag_icb.csv</t>
+  </si>
+  <si>
+    <t>requires additional bespoke grouping using ref_snomed_mh_ct.csv file</t>
+  </si>
+  <si>
+    <t>extracted to data folder - 111_sympt_icb.csv</t>
+  </si>
+  <si>
+    <t>extracted to data folder - 111_freqfly_icb.csv</t>
   </si>
 </sst>
 </file>
@@ -925,12 +943,12 @@
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -950,26 +968,38 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>145</v>
+        <v>144</v>
+      </c>
+      <c r="D8" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>149</v>
+      </c>
+      <c r="D9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E9" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
@@ -979,33 +1009,33 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B14" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B15" s="4"/>
       <c r="G15" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D16" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" t="s">
         <v>27</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>28</v>
       </c>
-      <c r="F16" t="s">
-        <v>29</v>
-      </c>
       <c r="G16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
@@ -1013,25 +1043,25 @@
         <v>4</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E17" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F17" s="5" t="s">
-        <v>31</v>
-      </c>
       <c r="G17" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
@@ -1039,25 +1069,25 @@
         <v>3</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F18" s="5" t="s">
-        <v>31</v>
-      </c>
       <c r="G18" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="1:9" s="5" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
@@ -1065,10 +1095,10 @@
         <v>5</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" spans="1:9" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
@@ -1076,56 +1106,56 @@
         <v>6</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="F20" s="5" t="s">
-        <v>141</v>
-      </c>
       <c r="G20" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="21" spans="1:9" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="B21" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E21" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="G21" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G21" s="5" t="s">
-        <v>144</v>
-      </c>
       <c r="H21" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1149,51 +1179,61 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{835B9890-ED73-4CF5-BE95-2A8A5BAE7287}">
   <dimension ref="A2:C18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="38.7265625" customWidth="1"/>
+    <col min="3" max="3" width="32.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>147</v>
+        <v>146</v>
+      </c>
+      <c r="C7" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B11" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -1204,7 +1244,7 @@
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -1212,7 +1252,7 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
@@ -1220,20 +1260,20 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1251,637 +1291,637 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B38" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="41" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B43" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B44" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="45" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B46" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="48" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B48" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B49" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B50" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="52" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B52" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="53" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B53" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="54" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="55" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B55" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="56" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B56" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="57" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="58" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="59" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B59" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="60" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="61" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="63" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="64" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="65" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="71" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B71" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="72" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B72" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="74" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B74" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="75" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B75" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="76" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B76" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="77" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="78" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="79" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B81" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="82" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B82" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="83" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B83" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="85" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B85" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="86" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B86" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="87" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B87" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="88" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B88" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="89" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B89" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="90" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B90" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="91" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B91" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="92" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B92" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="93" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B93" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="94" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B94" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="96" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B96" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B97" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B98" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B99" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B100" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B101" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="102" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B102" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="103" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B103" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="104" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B104" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="105" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B105" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="107" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B107" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="108" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B108" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="109" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B109" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="110" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B110" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="111" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B111" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="112" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B112" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="113" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B113" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="114" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B114" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="115" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B115" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="116" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B116" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="118" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B118" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="119" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B119" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="120" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B120" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="121" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B121" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="122" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B122" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="123" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B123" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="124" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B124" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="125" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B125" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="126" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B126" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="127" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B127" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="129" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B129" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="130" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B130" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="131" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B131" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="132" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B132" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="133" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B133" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="134" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B134" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="135" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B135" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="136" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B136" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="137" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B137" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="138" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B138" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="140" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B140" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="141" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B141" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="143" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B143" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added few more notes to metric descriptions
</commit_message>
<xml_diff>
--- a/data/cqc_metrics.xlsx
+++ b/data/cqc_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/andrew_hood_mlcsu_nhs_uk/Documents/Working Projects/ad-hoc/CQC SOC report/repo/cqc_soc/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="114_{98E47C94-B35C-48A9-87FF-0894DDAB52FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15380AE6-8203-4C5A-979E-A8E01706C37F}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="114_{98E47C94-B35C-48A9-87FF-0894DDAB52FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F67C7BB4-3E50-4E93-95B5-CBBE653A3A03}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11000" activeTab="1" xr2:uid="{E0173AC4-6F6F-4158-8A16-D04BBE4744E4}"/>
+    <workbookView xWindow="-28920" yWindow="10620" windowWidth="29040" windowHeight="15840" xr2:uid="{E0173AC4-6F6F-4158-8A16-D04BBE4744E4}"/>
   </bookViews>
   <sheets>
     <sheet name="UEC" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="159">
   <si>
     <t>% MH arriving by ambulance/self</t>
   </si>
@@ -500,13 +500,28 @@
   </si>
   <si>
     <t>extracted to data folder - 111_freqfly_icb.csv</t>
+  </si>
+  <si>
+    <t>field = "arrival_mode"</t>
+  </si>
+  <si>
+    <t>field  = "mhsds_flag"</t>
+  </si>
+  <si>
+    <t>field  = "mh_snomed"</t>
+  </si>
+  <si>
+    <t>field = "disch_dest"</t>
+  </si>
+  <si>
+    <t>ED (EC_Department_Type = 1) and UCC/WIC (EC_Department_Type = 3/4) to be done separately</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -561,6 +576,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -583,7 +605,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -598,6 +620,11 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -933,7 +960,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E043F9F0-0DBA-4E8F-9109-A6A749EE8BC1}">
-  <dimension ref="A2:I23"/>
+  <dimension ref="A2:I26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="15.81640625" customWidth="1"/>
@@ -941,181 +968,146 @@
     <col min="4" max="6" width="38.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B4" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B5" s="10"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
+      <c r="D7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B6" s="2" t="s">
+      <c r="D8" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B9" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
+      <c r="D9" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
+      <c r="D10" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B11" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D11" s="9" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
+    <row r="12" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B12" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D12" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E12" s="9" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
+    <row r="13" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B13" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D13" s="9" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B13" s="1" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B14" s="4" t="s">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B17" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B15" s="4"/>
-      <c r="G15" s="7" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B18" s="4"/>
+      <c r="G18" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="D16" t="s">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D19" t="s">
         <v>26</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E19" t="s">
         <v>27</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F19" t="s">
         <v>28</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G19" t="s">
         <v>32</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H19" t="s">
         <v>31</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I19" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B17" s="5" t="s">
+    <row r="20" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B20" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B18" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" s="5" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="B19" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
-      <c r="B20" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>140</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>143</v>
@@ -1127,21 +1119,21 @@
         <v>143</v>
       </c>
     </row>
-    <row r="21" spans="1:9" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" s="5" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B21" s="5" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D21" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E21" s="6" t="s">
-        <v>141</v>
-      </c>
       <c r="F21" s="5" t="s">
-        <v>142</v>
+        <v>30</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>143</v>
@@ -1153,22 +1145,85 @@
         <v>143</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+    <row r="22" spans="1:9" s="5" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="B22" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="B23" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="B24" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>20</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="D17" r:id="rId1" xr:uid="{11D6067B-A8E8-45DB-B183-F9A149027B92}"/>
-    <hyperlink ref="E17" r:id="rId2" xr:uid="{171B83D9-6216-4E69-B2EA-9CBC19E4A36D}"/>
-    <hyperlink ref="D18" r:id="rId3" xr:uid="{D42BD446-88BF-4F5A-A6A2-EAF9494FF80D}"/>
-    <hyperlink ref="E18" r:id="rId4" xr:uid="{091DCC6B-C431-46F9-8CD0-8CBE1F8127D5}"/>
-    <hyperlink ref="D20" r:id="rId5" xr:uid="{CAF6641D-1BEB-46D7-A18F-FA3FA25615E3}"/>
-    <hyperlink ref="E20" r:id="rId6" xr:uid="{60AD5DC8-5870-4485-9449-19048E8CCE84}"/>
-    <hyperlink ref="D21" r:id="rId7" xr:uid="{654D7616-7933-463E-A9B8-5C1D1C5C56E2}"/>
-    <hyperlink ref="E21" r:id="rId8" xr:uid="{23777C45-1E6F-4AD0-A9FC-E7A425AFC12B}"/>
+    <hyperlink ref="D20" r:id="rId1" xr:uid="{11D6067B-A8E8-45DB-B183-F9A149027B92}"/>
+    <hyperlink ref="E20" r:id="rId2" xr:uid="{171B83D9-6216-4E69-B2EA-9CBC19E4A36D}"/>
+    <hyperlink ref="D21" r:id="rId3" xr:uid="{D42BD446-88BF-4F5A-A6A2-EAF9494FF80D}"/>
+    <hyperlink ref="E21" r:id="rId4" xr:uid="{091DCC6B-C431-46F9-8CD0-8CBE1F8127D5}"/>
+    <hyperlink ref="D23" r:id="rId5" xr:uid="{CAF6641D-1BEB-46D7-A18F-FA3FA25615E3}"/>
+    <hyperlink ref="E23" r:id="rId6" xr:uid="{60AD5DC8-5870-4485-9449-19048E8CCE84}"/>
+    <hyperlink ref="D24" r:id="rId7" xr:uid="{654D7616-7933-463E-A9B8-5C1D1C5C56E2}"/>
+    <hyperlink ref="E24" r:id="rId8" xr:uid="{23777C45-1E6F-4AD0-A9FC-E7A425AFC12B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>

</xml_diff>